<commit_message>
modified:   catalog.xlsx 	new file:   images/1f.png
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>name</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t>test</t>
+  </si>
+  <si>
+    <t>images/1f.png</t>
   </si>
 </sst>
 </file>
@@ -95,55 +98,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>207818</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>85210</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Рисунок 8"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6470074" y="180110"/>
-          <a:ext cx="207817" cy="265318"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -466,9 +420,11 @@
       <c r="B2" t="s">
         <v>6</v>
       </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
modified:   catalog.xlsx 	new file:   images/2f.png 	new file:   images/3f.png 	new file:   images/4f.png 	new file:   images/5f.png 	new file:   images/6f.png 	new file:   images/7f.png
</commit_message>
<xml_diff>
--- a/catalog.xlsx
+++ b/catalog.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UNIKABOT\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9252"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264"/>
   </bookViews>
   <sheets>
-    <sheet name="Catalog" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>name</t>
   </si>
@@ -39,21 +39,110 @@
     <t>photo4</t>
   </si>
   <si>
-    <t>testing</t>
-  </si>
-  <si>
-    <t>test</t>
+    <t>Vanille Fraise</t>
+  </si>
+  <si>
+    <t>Summer Love = Candy Love</t>
+  </si>
+  <si>
+    <t>Limelight</t>
+  </si>
+  <si>
+    <t>Polar Bear</t>
+  </si>
+  <si>
+    <t>Phantom</t>
+  </si>
+  <si>
+    <t>Summer Breeze</t>
+  </si>
+  <si>
+    <t>Sugar Rash</t>
+  </si>
+  <si>
+    <t>Pink and Rose</t>
+  </si>
+  <si>
+    <t>Magical Sweet Summer</t>
+  </si>
+  <si>
+    <t>Samarskaya Lidia=Framboisine</t>
+  </si>
+  <si>
+    <t>Ванила Фрайз. Высота: 1,8 - 2,2 м. Соцветие: 35 - 40 см.</t>
+  </si>
+  <si>
+    <t>Самэр лов = Кэнди лов. Высота: 1,0 - 1,3 м. Соцветие: 25 - 35 см.</t>
+  </si>
+  <si>
+    <t>Лаймлайт. Высота: 1,8 - 2,2 м. Соцветие: 25 - 35 см.</t>
+  </si>
+  <si>
+    <t>Полярный Медведь. Высота: 1,8 - 2,0 м. Соцветие: 35 - 40 см.</t>
+  </si>
+  <si>
+    <t>Фантом. Высота: 1,8 - 2,5 м. Соцветие: 35 - 45 см.</t>
+  </si>
+  <si>
+    <t>Самер Бриз. Высота: 0,9 - 1,1 м. Соцветие: 20 - 25 см.</t>
+  </si>
+  <si>
+    <t>Шуга Раш. Высота: 1,2 - 1,5 м. Соцветие: 20 - 30 см.</t>
+  </si>
+  <si>
+    <t>Пинк энд Роуз. Высота: 1,2 - 1,5 м. Соцветие: 20 - 30 см.</t>
+  </si>
+  <si>
+    <t>Мэджикал Свит Самэр. Высота: 1,0 -1,2 м. Соцветие: 20 - 25 см.</t>
+  </si>
+  <si>
+    <t>Самарская Лидия. Высота: 0,8 - 1,1 м. Соцветие: 25 - 30 см.</t>
   </si>
   <si>
     <t>images/1f.png</t>
+  </si>
+  <si>
+    <t>images/2f.png</t>
+  </si>
+  <si>
+    <t>images/3f.png</t>
+  </si>
+  <si>
+    <t>images/4f.png</t>
+  </si>
+  <si>
+    <t>images/5f.png</t>
+  </si>
+  <si>
+    <t>images/6f.png</t>
+  </si>
+  <si>
+    <t>images/7f.png</t>
+  </si>
+  <si>
+    <t>images/8f.png</t>
+  </si>
+  <si>
+    <t>images/9f.png</t>
+  </si>
+  <si>
+    <t>images/10f.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -69,7 +158,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -77,12 +166,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -101,9 +208,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Стандартная">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -141,9 +248,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Стандартная">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -175,9 +282,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -209,9 +317,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Стандартная">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -385,46 +494,145 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="47.21875" customWidth="1"/>
-    <col min="2" max="2" width="47.109375" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" customWidth="1"/>
+    <col min="1" max="1" width="26.21875" customWidth="1"/>
+    <col min="2" max="2" width="56.109375" customWidth="1"/>
+    <col min="3" max="3" width="21.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>